<commit_message>
refactor: rewrite XLSX line items with dynamic rows, alternating styles, and remarks
- Remove fixed row assignments, write line items sequentially from row 31
- Add alternating white/blue styles with correct fills across all columns
- Add remark field to OfferLineItem (Bemerkung column C)
- Move Halteverbot/Umzugsmaterial details to remark instead of long descriptions
- Add orange header/total rows to items sheet with centered Nr/Anzahl/Volumen
- Parse quantity prefix from item names for Anzahl column
- Fix template: restore A:B fill styles, add missing merges for rows 34/36/40
- Fix template: signature line spacing in drawing
- Set docker containers to restart: always

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/offer_template.xlsx
+++ b/templates/offer_template.xlsx
@@ -226,7 +226,7 @@
     <numFmt numFmtId="170" formatCode="#,##0&quot; €&quot;;[RED]\-#,##0&quot; €&quot;"/>
     <numFmt numFmtId="171" formatCode="_-* #,##0.00&quot; €&quot;_-;\-* #,##0.00&quot; €&quot;_-;_-* \-??&quot; €&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -362,10 +362,22 @@
       <family val="0"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="0"/>
+    </font>
+    <font>
       <u val="single"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
       <family val="0"/>
     </font>
     <font>
@@ -395,6 +407,13 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="0"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -522,40 +541,44 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="83">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -563,59 +586,59 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -631,7 +654,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -639,171 +662,171 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -815,7 +838,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -823,17 +846,29 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
@@ -924,9 +959,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>704520</xdr:colOff>
+      <xdr:colOff>704160</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>185400</xdr:rowOff>
+      <xdr:rowOff>185040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -935,8 +970,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5563440" y="1796760"/>
-          <a:ext cx="2216160" cy="1058040"/>
+          <a:off x="5562720" y="1796760"/>
+          <a:ext cx="2215800" cy="1057680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1080,13 +1115,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>95400</xdr:colOff>
       <xdr:row>69</xdr:row>
-      <xdr:rowOff>128160</xdr:rowOff>
+      <xdr:rowOff>146160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>15120</xdr:colOff>
-      <xdr:row>121</xdr:row>
-      <xdr:rowOff>180360</xdr:rowOff>
+      <xdr:colOff>14760</xdr:colOff>
+      <xdr:row>117</xdr:row>
+      <xdr:rowOff>44640</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1096,7 +1131,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="95400" y="13700160"/>
-          <a:ext cx="5714640" cy="9957960"/>
+          <a:ext cx="5713560" cy="9042480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1775,7 +1810,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>______________________                                                        _________________________</a:t>
+            <a:t>_________________________                                   _______________________________________</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="de-DE" sz="1100" b="0" u="none" strike="noStrike">
@@ -1804,17 +1839,17 @@
             </a:tabLst>
           </a:pPr>
           <a:r>
-            <a:rPr lang="de-DE" sz="1100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:uFillTx/>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
+            <a:rPr lang="de-DE" sz="900" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>Datum, Unterschrift Kunde                                          Datum, Unterschrift Umzugsunternehmen</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="900" b="0" u="none" strike="noStrike">
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
@@ -1830,17 +1865,28 @@
             </a:tabLst>
           </a:pPr>
           <a:r>
-            <a:rPr lang="de-DE" sz="900" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:uFillTx/>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>Datum, Unterschrift Kunde                                                                               Datum, Unterschrift Umzugsunternehmen</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="900" b="0" u="none" strike="noStrike">
+            <a:rPr lang="de-DE" sz="1100" b="1" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>___________________________________________________________________________</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="de-DE" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
@@ -1882,17 +1928,6 @@
             </a:tabLst>
           </a:pPr>
           <a:r>
-            <a:rPr lang="de-DE" sz="1100" b="1" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:uFillTx/>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>___________________________________________________________________________</a:t>
-          </a:r>
-          <a:r>
             <a:rPr lang="de-DE" sz="1100" b="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
@@ -1927,7 +1962,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t> </a:t>
+            <a:t>Der Auftrag wurde ordnungsgemäß nach Kostenvoranschlag  </a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -1979,7 +2014,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>Der Auftrag wurde ordnungsgemäß nach Kostenvoranschlag  </a:t>
+            <a:t>durchgeführt am:  ______________________ </a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -2031,7 +2066,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>durchgeführt am:  ______________________ </a:t>
+            <a:t> </a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -2161,7 +2196,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t> </a:t>
+            <a:t>_______________________                                   _____________________________________ </a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -2179,58 +2214,6 @@
             </a:tabLst>
           </a:pPr>
           <a:r>
-            <a:rPr lang="de-DE" sz="1100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:uFillTx/>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
-            <a:effectLst/>
-            <a:uFillTx/>
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr defTabSz="914400">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:tabLst>
-              <a:tab algn="l" pos="0"/>
-            </a:tabLst>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="de-DE" sz="1100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:uFillTx/>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>______________________                                                             ______________________ </a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
-            <a:effectLst/>
-            <a:uFillTx/>
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr defTabSz="914400">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:tabLst>
-              <a:tab algn="l" pos="0"/>
-            </a:tabLst>
-          </a:pPr>
-          <a:r>
             <a:rPr lang="de-DE" sz="900" b="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
@@ -2239,7 +2222,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>Datum, Unterschrift Kunde                                                                                     Datum, Unterschrift Umzugsunternehmen</a:t>
+            <a:t>Datum, Unterschrift Kunde                                          Datum, Unterschrift Umzugsunternehmen</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="900" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -2275,9 +2258,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>545760</xdr:colOff>
+      <xdr:colOff>545400</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>38880</xdr:rowOff>
+      <xdr:rowOff>38520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2290,8 +2273,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5201280" y="371520"/>
-          <a:ext cx="2419560" cy="1575000"/>
+          <a:off x="5200560" y="371520"/>
+          <a:ext cx="2419200" cy="1574640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2480,896 +2463,896 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:N56"/>
   <sheetFormatPr defaultColWidth="11.4296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.72"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="4" min="4" style="0" width="53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="5.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27.72"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="4" min="4" style="1" width="53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="20.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="4"/>
-      <c r="J3" s="0" t="str">
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="5"/>
+      <c r="J3" s="1" t="str">
         <f aca="false">A16</f>
         <v>Unverbindlicher Kostenvoranschlag 2026-132</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I4" s="0" t="str">
+      <c r="I4" s="1" t="str">
         <f aca="false">A8</f>
         <v>Herrn</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="I5" s="0" t="str">
+      <c r="B5" s="6"/>
+      <c r="I5" s="1" t="str">
         <f aca="false">A9</f>
         <v>Horst Lindenthal</v>
       </c>
-      <c r="K5" s="0" t="str">
+      <c r="K5" s="1" t="str">
         <f aca="false">F18</f>
         <v>delphinchris007@web.de</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="I6" s="0" t="str">
+      <c r="B6" s="6"/>
+      <c r="I6" s="1" t="str">
         <f aca="false">A17</f>
         <v>Auftragsdatum: </v>
       </c>
-      <c r="J6" s="6" t="str">
+      <c r="J6" s="7" t="str">
         <f aca="false">B17</f>
         <v>KW 13-14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I7" s="7" t="str">
+      <c r="I7" s="8" t="str">
         <f aca="false">A18</f>
         <v>Kundentelefonnr.: </v>
       </c>
-      <c r="J7" s="8" t="str">
+      <c r="J7" s="9" t="str">
         <f aca="false">B18</f>
         <v>01746555333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="0" t="str">
+      <c r="I9" s="1" t="str">
         <f aca="false">A25</f>
         <v>Beladestelle:</v>
       </c>
-      <c r="L9" s="0" t="str">
+      <c r="L9" s="1" t="str">
         <f aca="false">F25</f>
         <v>Entladestelle:</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="I10" s="0" t="str">
+      <c r="B10" s="8"/>
+      <c r="I10" s="1" t="str">
         <f aca="false">A26</f>
         <v>Schlickumerstr. 15A</v>
       </c>
-      <c r="L10" s="0" t="str">
+      <c r="L10" s="1" t="str">
         <f aca="false">F26</f>
         <v>Weinhagenstr. 9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="7"/>
-      <c r="I11" s="0" t="str">
+      <c r="B11" s="8"/>
+      <c r="I11" s="1" t="str">
         <f aca="false">A27</f>
         <v>31157 Sarstedt</v>
       </c>
-      <c r="L11" s="9" t="str">
+      <c r="L11" s="10" t="str">
         <f aca="false">F27</f>
         <v>31135 Hildesheim</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I12" s="0" t="str">
+      <c r="I12" s="1" t="str">
         <f aca="false">A28</f>
         <v>2OG mit Fahrstuhl</v>
       </c>
-      <c r="L12" s="0" t="str">
+      <c r="L12" s="1" t="str">
         <f aca="false">F28</f>
         <v>1 OG </v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G14" s="10" t="n">
+      <c r="G14" s="11" t="n">
         <f aca="true">(TODAY())</f>
-        <v>46077</v>
-      </c>
-      <c r="I14" s="0" t="str">
+        <v>46078</v>
+      </c>
+      <c r="I14" s="1" t="str">
         <f aca="false">A29</f>
         <v>Umzugspauschale 15 m³</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I15" s="11" t="s">
+      <c r="I15" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11" t="s">
+      <c r="J15" s="12"/>
+      <c r="K15" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="L15" s="12"/>
-      <c r="M15" s="13" t="s">
+      <c r="L15" s="13"/>
+      <c r="M15" s="14" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="I16" s="16" t="str">
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="I16" s="17" t="str">
         <f aca="false">A31</f>
         <v>De/Montage</v>
       </c>
-      <c r="J16" s="16"/>
-      <c r="K16" s="17" t="n">
+      <c r="J16" s="17"/>
+      <c r="K16" s="18" t="n">
         <f aca="false">C31</f>
         <v>0</v>
       </c>
-      <c r="L16" s="18"/>
-      <c r="M16" s="18" t="n">
+      <c r="L16" s="19"/>
+      <c r="M16" s="19" t="n">
         <f aca="false">E31</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="I17" s="20" t="str">
+      <c r="C17" s="20"/>
+      <c r="I17" s="21" t="str">
         <f aca="false">A32</f>
         <v>Halteverbotszone</v>
       </c>
-      <c r="J17" s="20"/>
-      <c r="K17" s="21" t="str">
+      <c r="J17" s="21"/>
+      <c r="K17" s="22" t="str">
         <f aca="false">C32</f>
         <v> Entladestelle</v>
       </c>
-      <c r="L17" s="22"/>
-      <c r="M17" s="22" t="n">
+      <c r="L17" s="23"/>
+      <c r="M17" s="23" t="n">
         <f aca="false">E32</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="8"/>
-      <c r="E18" s="24" t="s">
+      <c r="C18" s="9"/>
+      <c r="E18" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="F18" s="25" t="s">
+      <c r="F18" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="26"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="16" t="str">
+      <c r="G18" s="27"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="17" t="str">
         <f aca="false">A33</f>
         <v>Umzugsmaterial</v>
       </c>
-      <c r="J18" s="16"/>
-      <c r="K18" s="17" t="str">
+      <c r="J18" s="17"/>
+      <c r="K18" s="18" t="str">
         <f aca="false">C33</f>
         <v>Stretchfolie,Decken,Gurte</v>
       </c>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18" t="n">
+      <c r="L18" s="19"/>
+      <c r="M18" s="19" t="n">
         <f aca="false">E33</f>
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="28"/>
-      <c r="C19" s="8"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="I19" s="29" t="str">
+      <c r="B19" s="29"/>
+      <c r="C19" s="9"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="I19" s="30" t="str">
         <f aca="false">A34</f>
         <v>Verkauf Seidenpapier</v>
       </c>
-      <c r="J19" s="30"/>
-      <c r="K19" s="21" t="str">
+      <c r="J19" s="31"/>
+      <c r="K19" s="22" t="str">
         <f aca="false">C34</f>
         <v>500x750 </v>
       </c>
-      <c r="L19" s="22"/>
-      <c r="M19" s="22" t="n">
+      <c r="L19" s="23"/>
+      <c r="M19" s="23" t="n">
         <f aca="false">E34</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="31"/>
-      <c r="C20" s="31"/>
-      <c r="G20" s="32"/>
-      <c r="I20" s="16" t="str">
+      <c r="B20" s="32"/>
+      <c r="C20" s="32"/>
+      <c r="G20" s="33"/>
+      <c r="I20" s="17" t="str">
         <f aca="false">A35</f>
         <v>Verkauf U-Karton</v>
       </c>
-      <c r="J20" s="16"/>
-      <c r="K20" s="17" t="str">
+      <c r="J20" s="17"/>
+      <c r="K20" s="18" t="str">
         <f aca="false">C35</f>
         <v>590x318x328</v>
       </c>
-      <c r="L20" s="18"/>
-      <c r="M20" s="18" t="n">
+      <c r="L20" s="19"/>
+      <c r="M20" s="19" t="n">
         <f aca="false">E35</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I21" s="20" t="str">
+      <c r="I21" s="21" t="str">
         <f aca="false">A37</f>
         <v>Verleih Kleiderboxen</v>
       </c>
-      <c r="J21" s="20"/>
-      <c r="K21" s="21" t="str">
+      <c r="J21" s="21"/>
+      <c r="K21" s="22" t="str">
         <f aca="false">C36</f>
         <v>400x318x328</v>
       </c>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22" t="n">
+      <c r="L21" s="23"/>
+      <c r="M21" s="23" t="n">
         <f aca="false">E37</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="33" t="str">
+      <c r="I22" s="34" t="str">
         <f aca="false">A38</f>
         <v>Personal</v>
       </c>
-      <c r="J22" s="33"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="18" t="n">
+      <c r="J22" s="34"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="19" t="n">
         <f aca="false">E38</f>
         <v>3</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="20" t="str">
+      <c r="I23" s="21" t="str">
         <f aca="false">A39</f>
         <v>3,5t Transporter m. Koffer</v>
       </c>
-      <c r="J23" s="20"/>
-      <c r="K23" s="21" t="n">
+      <c r="J23" s="21"/>
+      <c r="K23" s="22" t="n">
         <f aca="false">C39</f>
         <v>0</v>
       </c>
-      <c r="L23" s="22"/>
-      <c r="M23" s="22" t="n">
+      <c r="L23" s="23"/>
+      <c r="M23" s="23" t="n">
         <f aca="false">E39</f>
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I24" s="16" t="str">
+      <c r="I24" s="17" t="str">
         <f aca="false">A41</f>
         <v>Transferfahrzeug</v>
       </c>
-      <c r="J24" s="16"/>
-      <c r="K24" s="17" t="n">
+      <c r="J24" s="17"/>
+      <c r="K24" s="18" t="n">
         <f aca="false">C41</f>
         <v>0</v>
       </c>
-      <c r="L24" s="18"/>
-      <c r="M24" s="18" t="n">
+      <c r="L24" s="19"/>
+      <c r="M24" s="19" t="n">
         <f aca="false">E41</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="34" t="s">
+      <c r="A25" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B25" s="34"/>
-      <c r="D25" s="35" t="s">
+      <c r="B25" s="35"/>
+      <c r="D25" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="F25" s="36" t="s">
+      <c r="F25" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="G25" s="36"/>
-      <c r="H25" s="36"/>
-      <c r="I25" s="37"/>
-      <c r="J25" s="37"/>
-      <c r="K25" s="21"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="22"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="38"/>
+      <c r="J25" s="38"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="23"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="38" t="str">
+      <c r="A26" s="39" t="str">
         <f aca="false">A10</f>
         <v>Schlickumerstr. 15A</v>
       </c>
-      <c r="B26" s="38"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="35"/>
-      <c r="F26" s="39" t="s">
+      <c r="B26" s="39"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="36"/>
+      <c r="F26" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="G26" s="39"/>
+      <c r="G26" s="40"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="38" t="str">
+      <c r="A27" s="39" t="str">
         <f aca="false">A11</f>
         <v>31157 Sarstedt</v>
       </c>
-      <c r="B27" s="38"/>
-      <c r="D27" s="35"/>
-      <c r="F27" s="40" t="s">
+      <c r="B27" s="39"/>
+      <c r="D27" s="36"/>
+      <c r="F27" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="G27" s="41"/>
-      <c r="H27" s="42"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="43"/>
     </row>
     <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="43" t="s">
+      <c r="A28" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="44"/>
-      <c r="D28" s="35"/>
-      <c r="F28" s="0" t="s">
+      <c r="B28" s="45"/>
+      <c r="D28" s="36"/>
+      <c r="F28" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G28" s="45"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="46"/>
-      <c r="J28" s="46"/>
-      <c r="K28" s="46"/>
-      <c r="L28" s="46"/>
-      <c r="M28" s="46"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="47"/>
+      <c r="J28" s="47"/>
+      <c r="K28" s="47"/>
+      <c r="L28" s="47"/>
+      <c r="M28" s="47"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="47" t="s">
+      <c r="A29" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="47"/>
-      <c r="C29" s="47"/>
-      <c r="D29" s="47"/>
-      <c r="E29" s="47"/>
-      <c r="F29" s="47"/>
-      <c r="G29" s="47"/>
-      <c r="I29" s="46"/>
-      <c r="J29" s="46"/>
-      <c r="K29" s="46"/>
-      <c r="L29" s="46"/>
-      <c r="M29" s="46"/>
-      <c r="N29" s="48"/>
+      <c r="B29" s="48"/>
+      <c r="C29" s="48"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="48"/>
+      <c r="G29" s="48"/>
+      <c r="I29" s="47"/>
+      <c r="J29" s="47"/>
+      <c r="K29" s="47"/>
+      <c r="L29" s="47"/>
+      <c r="M29" s="47"/>
+      <c r="N29" s="49"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="49" t="s">
+      <c r="A30" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="B30" s="49"/>
-      <c r="C30" s="50" t="s">
+      <c r="B30" s="50"/>
+      <c r="C30" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="27"/>
-      <c r="E30" s="51" t="s">
+      <c r="D30" s="28"/>
+      <c r="E30" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="F30" s="35" t="s">
+      <c r="F30" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="G30" s="51" t="s">
+      <c r="G30" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="I30" s="46"/>
-      <c r="J30" s="46"/>
-      <c r="K30" s="46"/>
-      <c r="L30" s="46"/>
-      <c r="M30" s="46"/>
-      <c r="N30" s="52"/>
+      <c r="I30" s="47"/>
+      <c r="J30" s="47"/>
+      <c r="K30" s="47"/>
+      <c r="L30" s="47"/>
+      <c r="M30" s="47"/>
+      <c r="N30" s="53"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="53" t="s">
+      <c r="A31" s="54" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="53"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="55"/>
-      <c r="E31" s="55" t="n">
+      <c r="B31" s="54"/>
+      <c r="C31" s="55"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="F31" s="56" t="n">
+      <c r="F31" s="57" t="n">
         <v>50</v>
       </c>
-      <c r="G31" s="56" t="n">
+      <c r="G31" s="57" t="n">
         <f aca="false">IF(E31="", 0, F31*E31)</f>
         <v>0</v>
       </c>
-      <c r="N31" s="57"/>
+      <c r="N31" s="58"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="58" t="s">
+      <c r="A32" s="59" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="58"/>
-      <c r="C32" s="59" t="s">
+      <c r="B32" s="59"/>
+      <c r="C32" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="D32" s="60"/>
-      <c r="E32" s="60" t="n">
+      <c r="D32" s="61"/>
+      <c r="E32" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="F32" s="61" t="n">
+      <c r="F32" s="62" t="n">
         <v>100</v>
       </c>
-      <c r="G32" s="61" t="n">
+      <c r="G32" s="62" t="n">
         <f aca="false">IF(E32="", 0, F32*E32)</f>
         <v>0</v>
       </c>
-      <c r="I32" s="62"/>
-      <c r="J32" s="62"/>
-      <c r="K32" s="62"/>
-      <c r="L32" s="62"/>
-      <c r="M32" s="62"/>
+      <c r="I32" s="63"/>
+      <c r="J32" s="63"/>
+      <c r="K32" s="63"/>
+      <c r="L32" s="63"/>
+      <c r="M32" s="63"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="53" t="s">
+      <c r="A33" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="53"/>
-      <c r="C33" s="54" t="s">
+      <c r="B33" s="54"/>
+      <c r="C33" s="55" t="s">
         <v>33</v>
       </c>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55" t="n">
+      <c r="D33" s="56"/>
+      <c r="E33" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F33" s="56" t="n">
+      <c r="F33" s="57" t="n">
         <v>30</v>
       </c>
-      <c r="G33" s="56" t="n">
+      <c r="G33" s="57" t="n">
         <f aca="false">IF(E33="", 0, F33*E33)</f>
         <v>30</v>
       </c>
-      <c r="I33" s="62"/>
-      <c r="J33" s="62"/>
-      <c r="K33" s="62"/>
-      <c r="L33" s="62"/>
-      <c r="M33" s="62"/>
+      <c r="I33" s="63"/>
+      <c r="J33" s="63"/>
+      <c r="K33" s="63"/>
+      <c r="L33" s="63"/>
+      <c r="M33" s="63"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="63" t="s">
+      <c r="A34" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="B34" s="63"/>
-      <c r="C34" s="59" t="s">
+      <c r="B34" s="64"/>
+      <c r="C34" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="D34" s="60"/>
-      <c r="E34" s="60" t="n">
+      <c r="D34" s="61"/>
+      <c r="E34" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="F34" s="61" t="n">
+      <c r="F34" s="62" t="n">
         <v>5</v>
       </c>
-      <c r="G34" s="61" t="n">
+      <c r="G34" s="62" t="n">
         <f aca="false">IF(E34="", 0, F34*E34)</f>
         <v>0</v>
       </c>
-      <c r="I34" s="62"/>
-      <c r="J34" s="62"/>
-      <c r="K34" s="62"/>
-      <c r="L34" s="62"/>
-      <c r="M34" s="62"/>
+      <c r="I34" s="63"/>
+      <c r="J34" s="63"/>
+      <c r="K34" s="63"/>
+      <c r="L34" s="63"/>
+      <c r="M34" s="63"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="53" t="s">
+      <c r="A35" s="54" t="s">
         <v>36</v>
       </c>
-      <c r="B35" s="53"/>
-      <c r="C35" s="54" t="s">
+      <c r="B35" s="54"/>
+      <c r="C35" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55" t="n">
+      <c r="D35" s="56"/>
+      <c r="E35" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="F35" s="56" t="n">
+      <c r="F35" s="57" t="n">
         <v>2.1</v>
       </c>
-      <c r="G35" s="56" t="n">
+      <c r="G35" s="57" t="n">
         <f aca="false">IF(E35="", 0, F35*E35)</f>
         <v>0</v>
       </c>
-      <c r="I35" s="62"/>
-      <c r="J35" s="62"/>
-      <c r="K35" s="62"/>
-      <c r="L35" s="62"/>
-      <c r="M35" s="62"/>
+      <c r="I35" s="63"/>
+      <c r="J35" s="63"/>
+      <c r="K35" s="63"/>
+      <c r="L35" s="63"/>
+      <c r="M35" s="63"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="64" t="s">
+      <c r="A36" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="64"/>
-      <c r="C36" s="59" t="s">
+      <c r="B36" s="65"/>
+      <c r="C36" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="D36" s="60"/>
-      <c r="E36" s="60" t="n">
+      <c r="D36" s="61"/>
+      <c r="E36" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="61" t="n">
+      <c r="F36" s="62" t="n">
         <v>2.2</v>
       </c>
-      <c r="G36" s="61" t="n">
+      <c r="G36" s="62" t="n">
         <f aca="false">IF(E36="", 0, F36*E36)</f>
         <v>0</v>
       </c>
-      <c r="I36" s="62"/>
-      <c r="J36" s="62"/>
-      <c r="K36" s="62"/>
-      <c r="L36" s="62"/>
-      <c r="M36" s="62"/>
+      <c r="I36" s="63"/>
+      <c r="J36" s="63"/>
+      <c r="K36" s="63"/>
+      <c r="L36" s="63"/>
+      <c r="M36" s="63"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="53" t="s">
+      <c r="A37" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="B37" s="53"/>
-      <c r="C37" s="65" t="s">
+      <c r="B37" s="54"/>
+      <c r="C37" s="66" t="s">
         <v>41</v>
       </c>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55" t="n">
+      <c r="D37" s="56"/>
+      <c r="E37" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="F37" s="56" t="n">
+      <c r="F37" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="G37" s="56" t="n">
+      <c r="G37" s="57" t="n">
         <f aca="false">IF(E37="", 0, F37*E37)</f>
         <v>0</v>
       </c>
-      <c r="I37" s="62"/>
-      <c r="J37" s="62"/>
-      <c r="K37" s="62"/>
-      <c r="L37" s="62"/>
-      <c r="M37" s="62"/>
+      <c r="I37" s="63"/>
+      <c r="J37" s="63"/>
+      <c r="K37" s="63"/>
+      <c r="L37" s="63"/>
+      <c r="M37" s="63"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="66" t="s">
+      <c r="A38" s="67" t="s">
         <v>42</v>
       </c>
-      <c r="B38" s="66"/>
-      <c r="C38" s="59"/>
-      <c r="D38" s="60" t="s">
+      <c r="B38" s="67"/>
+      <c r="C38" s="60"/>
+      <c r="D38" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="E38" s="60" t="n">
+      <c r="E38" s="61" t="n">
         <v>3</v>
       </c>
-      <c r="F38" s="61" t="n">
+      <c r="F38" s="62" t="n">
         <v>28</v>
       </c>
-      <c r="G38" s="61" t="n">
+      <c r="G38" s="62" t="n">
         <f aca="false">IF(E38="", 0, F38*E38*J50)</f>
         <v>0</v>
       </c>
-      <c r="I38" s="62"/>
-      <c r="J38" s="62"/>
-      <c r="K38" s="62"/>
-      <c r="L38" s="62"/>
-      <c r="M38" s="62"/>
+      <c r="I38" s="63"/>
+      <c r="J38" s="63"/>
+      <c r="K38" s="63"/>
+      <c r="L38" s="63"/>
+      <c r="M38" s="63"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="53" t="s">
+      <c r="A39" s="54" t="s">
         <v>44</v>
       </c>
-      <c r="B39" s="53"/>
-      <c r="C39" s="54"/>
-      <c r="D39" s="55"/>
-      <c r="E39" s="55" t="n">
+      <c r="B39" s="54"/>
+      <c r="C39" s="55"/>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="F39" s="56" t="n">
+      <c r="F39" s="57" t="n">
         <v>60</v>
       </c>
-      <c r="G39" s="56" t="n">
+      <c r="G39" s="57" t="n">
         <f aca="false">IF(E39="", 0, F39*E39)</f>
         <v>60</v>
       </c>
-      <c r="I39" s="62"/>
-      <c r="J39" s="62"/>
-      <c r="K39" s="62"/>
-      <c r="L39" s="62"/>
-      <c r="M39" s="62"/>
-      <c r="N39" s="52"/>
+      <c r="I39" s="63"/>
+      <c r="J39" s="63"/>
+      <c r="K39" s="63"/>
+      <c r="L39" s="63"/>
+      <c r="M39" s="63"/>
+      <c r="N39" s="53"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="64" t="s">
+      <c r="A40" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="B40" s="64"/>
-      <c r="C40" s="59"/>
-      <c r="D40" s="60"/>
-      <c r="E40" s="60" t="n">
+      <c r="B40" s="65"/>
+      <c r="C40" s="60"/>
+      <c r="D40" s="61"/>
+      <c r="E40" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="F40" s="61" t="n">
+      <c r="F40" s="62" t="n">
         <v>300</v>
       </c>
-      <c r="G40" s="61" t="n">
+      <c r="G40" s="62" t="n">
         <f aca="false">IF(E40="", 0, F40*E40)</f>
         <v>0</v>
       </c>
-      <c r="I40" s="62"/>
-      <c r="J40" s="62"/>
-      <c r="K40" s="62"/>
-      <c r="L40" s="62"/>
-      <c r="M40" s="62"/>
-      <c r="N40" s="52"/>
+      <c r="I40" s="63"/>
+      <c r="J40" s="63"/>
+      <c r="K40" s="63"/>
+      <c r="L40" s="63"/>
+      <c r="M40" s="63"/>
+      <c r="N40" s="53"/>
     </row>
     <row r="41" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="53" t="s">
+      <c r="A41" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="B41" s="53"/>
-      <c r="C41" s="54"/>
-      <c r="D41" s="55" t="s">
+      <c r="B41" s="54"/>
+      <c r="C41" s="55"/>
+      <c r="D41" s="56" t="s">
         <v>47</v>
       </c>
-      <c r="E41" s="55" t="n">
+      <c r="E41" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="56" t="n">
+      <c r="F41" s="57" t="n">
         <v>45</v>
       </c>
-      <c r="G41" s="56" t="n">
+      <c r="G41" s="57" t="n">
         <f aca="false">IF(E41="", 0, F41*E41)</f>
         <v>0</v>
       </c>
-      <c r="I41" s="62"/>
-      <c r="J41" s="62"/>
-      <c r="K41" s="62"/>
-      <c r="L41" s="62"/>
-      <c r="M41" s="62"/>
-      <c r="N41" s="60"/>
+      <c r="I41" s="63"/>
+      <c r="J41" s="63"/>
+      <c r="K41" s="63"/>
+      <c r="L41" s="63"/>
+      <c r="M41" s="63"/>
+      <c r="N41" s="61"/>
     </row>
     <row r="42" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="58" t="s">
+      <c r="A42" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="B42" s="58"/>
-      <c r="C42" s="59"/>
-      <c r="D42" s="60" t="s">
+      <c r="B42" s="59"/>
+      <c r="C42" s="60"/>
+      <c r="D42" s="61" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="60" t="n">
+      <c r="E42" s="61" t="n">
         <v>1</v>
       </c>
-      <c r="F42" s="61" t="n">
+      <c r="F42" s="62" t="n">
         <v>30</v>
       </c>
-      <c r="G42" s="61" t="n">
+      <c r="G42" s="62" t="n">
         <f aca="false">IF(E42="", 0, F42*E42)</f>
         <v>30</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="67"/>
-      <c r="D43" s="68"/>
-      <c r="E43" s="68"/>
-      <c r="F43" s="68"/>
-      <c r="G43" s="68"/>
+      <c r="A43" s="8"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="68"/>
+      <c r="D43" s="69"/>
+      <c r="E43" s="69"/>
+      <c r="F43" s="69"/>
+      <c r="G43" s="69"/>
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7"/>
-      <c r="C44" s="69" t="s">
+      <c r="A44" s="8"/>
+      <c r="C44" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="D44" s="68"/>
-      <c r="E44" s="70"/>
-      <c r="F44" s="70"/>
-      <c r="G44" s="71" t="n">
+      <c r="D44" s="69"/>
+      <c r="E44" s="71"/>
+      <c r="F44" s="71"/>
+      <c r="G44" s="72" t="n">
         <f aca="false">G31+G32+G33+G34+G35+G37+G38+G39+G41+G42+G40</f>
         <v>120</v>
       </c>
-      <c r="J44" s="52"/>
-    </row>
-    <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7"/>
-      <c r="C45" s="69" t="s">
+      <c r="J44" s="53"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="8"/>
+      <c r="C45" s="70" t="s">
         <v>50</v>
       </c>
-      <c r="D45" s="68"/>
-      <c r="E45" s="70"/>
-      <c r="F45" s="70"/>
-      <c r="G45" s="71" t="n">
+      <c r="D45" s="69"/>
+      <c r="E45" s="71"/>
+      <c r="F45" s="71"/>
+      <c r="G45" s="72" t="n">
         <f aca="false">G44*19%</f>
         <v>22.8</v>
       </c>
-      <c r="J45" s="52"/>
-      <c r="M45" s="72"/>
+      <c r="J45" s="53"/>
+      <c r="M45" s="73"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C46" s="0" t="s">
+      <c r="C46" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E46" s="73"/>
-      <c r="F46" s="73"/>
-      <c r="G46" s="74" t="n">
+      <c r="E46" s="74"/>
+      <c r="F46" s="74"/>
+      <c r="G46" s="75" t="n">
         <f aca="false">G44+G45</f>
         <v>142.8</v>
       </c>
-      <c r="J46" s="52"/>
-      <c r="M46" s="72"/>
+      <c r="J46" s="53"/>
+      <c r="M46" s="73"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J47" s="52"/>
-      <c r="M47" s="72"/>
+      <c r="J47" s="53"/>
+      <c r="M47" s="73"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="46"/>
-      <c r="B48" s="46"/>
-      <c r="C48" s="46"/>
-      <c r="D48" s="46"/>
-      <c r="E48" s="46"/>
-      <c r="F48" s="46"/>
-      <c r="G48" s="46"/>
-      <c r="J48" s="52"/>
-      <c r="M48" s="72"/>
+      <c r="A48" s="47"/>
+      <c r="B48" s="47"/>
+      <c r="C48" s="47"/>
+      <c r="D48" s="47"/>
+      <c r="E48" s="47"/>
+      <c r="F48" s="47"/>
+      <c r="G48" s="47"/>
+      <c r="J48" s="53"/>
+      <c r="M48" s="73"/>
     </row>
     <row r="49" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="46"/>
-      <c r="B49" s="46"/>
-      <c r="C49" s="46"/>
-      <c r="D49" s="46"/>
-      <c r="E49" s="46"/>
-      <c r="F49" s="46"/>
-      <c r="G49" s="46"/>
-      <c r="J49" s="52"/>
-      <c r="M49" s="72"/>
+      <c r="A49" s="47"/>
+      <c r="B49" s="47"/>
+      <c r="C49" s="47"/>
+      <c r="D49" s="47"/>
+      <c r="E49" s="47"/>
+      <c r="F49" s="47"/>
+      <c r="G49" s="47"/>
+      <c r="J49" s="53"/>
+      <c r="M49" s="73"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="46"/>
-      <c r="B50" s="46"/>
-      <c r="C50" s="46"/>
-      <c r="D50" s="46"/>
-      <c r="E50" s="46"/>
-      <c r="F50" s="46"/>
-      <c r="G50" s="46"/>
-      <c r="J50" s="75"/>
-      <c r="M50" s="76"/>
+      <c r="A50" s="47"/>
+      <c r="B50" s="47"/>
+      <c r="C50" s="47"/>
+      <c r="D50" s="47"/>
+      <c r="E50" s="47"/>
+      <c r="F50" s="47"/>
+      <c r="G50" s="47"/>
+      <c r="J50" s="76"/>
+      <c r="M50" s="77"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="46"/>
-      <c r="B51" s="46"/>
-      <c r="C51" s="46"/>
-      <c r="D51" s="46"/>
-      <c r="E51" s="46"/>
-      <c r="F51" s="46"/>
-      <c r="G51" s="46"/>
-      <c r="J51" s="52"/>
-      <c r="M51" s="76"/>
+      <c r="A51" s="47"/>
+      <c r="B51" s="47"/>
+      <c r="C51" s="47"/>
+      <c r="D51" s="47"/>
+      <c r="E51" s="47"/>
+      <c r="F51" s="47"/>
+      <c r="G51" s="47"/>
+      <c r="J51" s="53"/>
+      <c r="M51" s="77"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="46"/>
-      <c r="B52" s="46"/>
-      <c r="C52" s="46"/>
-      <c r="D52" s="46"/>
-      <c r="E52" s="46"/>
-      <c r="F52" s="46"/>
-      <c r="G52" s="46"/>
+      <c r="A52" s="47"/>
+      <c r="B52" s="47"/>
+      <c r="C52" s="47"/>
+      <c r="D52" s="47"/>
+      <c r="E52" s="47"/>
+      <c r="F52" s="47"/>
+      <c r="G52" s="47"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="46"/>
-      <c r="B53" s="46"/>
-      <c r="C53" s="46"/>
-      <c r="D53" s="46"/>
-      <c r="E53" s="46"/>
-      <c r="F53" s="46"/>
-      <c r="G53" s="46"/>
+      <c r="A53" s="47"/>
+      <c r="B53" s="47"/>
+      <c r="C53" s="47"/>
+      <c r="D53" s="47"/>
+      <c r="E53" s="47"/>
+      <c r="F53" s="47"/>
+      <c r="G53" s="47"/>
     </row>
     <row r="54" customFormat="false" ht="2.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="46"/>
-      <c r="B54" s="46"/>
-      <c r="C54" s="46"/>
-      <c r="D54" s="46"/>
-      <c r="E54" s="46"/>
-      <c r="F54" s="46"/>
-      <c r="G54" s="46"/>
+      <c r="A54" s="47"/>
+      <c r="B54" s="47"/>
+      <c r="C54" s="47"/>
+      <c r="D54" s="47"/>
+      <c r="E54" s="47"/>
+      <c r="F54" s="47"/>
+      <c r="G54" s="47"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="46"/>
-      <c r="B55" s="46"/>
-      <c r="C55" s="46"/>
-      <c r="D55" s="46"/>
-      <c r="E55" s="46"/>
-      <c r="F55" s="46"/>
-      <c r="G55" s="46"/>
-      <c r="J55" s="77"/>
+      <c r="A55" s="47"/>
+      <c r="B55" s="47"/>
+      <c r="C55" s="47"/>
+      <c r="D55" s="47"/>
+      <c r="E55" s="47"/>
+      <c r="F55" s="47"/>
+      <c r="G55" s="47"/>
+      <c r="J55" s="78"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="46"/>
-      <c r="B56" s="46"/>
-      <c r="C56" s="46"/>
-      <c r="D56" s="46"/>
-      <c r="E56" s="46"/>
-      <c r="F56" s="46"/>
-      <c r="G56" s="46"/>
+      <c r="A56" s="47"/>
+      <c r="B56" s="47"/>
+      <c r="C56" s="47"/>
+      <c r="D56" s="47"/>
+      <c r="E56" s="47"/>
+      <c r="F56" s="47"/>
+      <c r="G56" s="47"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
+  <mergeCells count="38">
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
@@ -3405,6 +3388,9 @@
     <mergeCell ref="A42:B42"/>
     <mergeCell ref="A48:G49"/>
     <mergeCell ref="A50:G56"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A40:B40"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E18" r:id="rId1" display="E-Mail: "/>

</xml_diff>

<commit_message>
feat: add € formatting to Einzelpreis and Gesamt Netto columns
- Einzelpreis shows € via number format, labor shows €/Stunde
- Gesamt Netto right-aligned with € number format
- Nettobetrag/Umsatzsteuer/Bruttobetrag right-aligned
- Center Einzelpreis header, remove accidental borders
- Remove unused Formula variant

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/offer_template.xlsx
+++ b/templates/offer_template.xlsx
@@ -216,7 +216,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy;@"/>
     <numFmt numFmtId="166" formatCode="[&lt;=9999999]###\-####;\(###&quot;) &quot;###\-####"/>
@@ -225,6 +225,7 @@
     <numFmt numFmtId="169" formatCode="_-* #,##0.00\ [$€-407]_-;\-* #,##0.00\ [$€-407]_-;_-* \-??\ [$€-407]_-;_-@_-"/>
     <numFmt numFmtId="170" formatCode="#,##0&quot; €&quot;;[RED]\-#,##0&quot; €&quot;"/>
     <numFmt numFmtId="171" formatCode="_-* #,##0.00&quot; €&quot;_-;\-* #,##0.00&quot; €&quot;_-;_-* \-??&quot; €&quot;_-;_-@_-"/>
+    <numFmt numFmtId="172" formatCode="#,##0.00&quot; €/Stunde&quot;"/>
   </numFmts>
   <fonts count="27">
     <font>
@@ -541,7 +542,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="87">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -687,7 +688,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -766,7 +767,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true" applyNumberFormat="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -786,7 +787,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true" applyNumberFormat="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -831,7 +832,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -843,7 +844,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="17" fillId="0" borderId="0" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -868,6 +869,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
feat: transporter line item (60€, editable), fix quantity parsing, update AGENT_API.md, archive resolved bug reports
Backend:
- Add Services.transporter flag + CompanyConfig.transporter_price (default 60€)
- Add transporter to build_line_items(), ServicePrices, format_services_display()
- Fix inquiry_builder quantity=1 hardcode — parse Nx prefix from item names
- Update submission/orchestrator paths to set transporter=true by default
- Remove 'Kartons werden vorzeitig geliefert...' sentence from offer_template.xlsx
- Update AGENT_API.md with api.aufraeumhelden.com base URL + agent credentials

Frontend (submodule):
- Add transporter checkbox to CreateInquiryModal (default on)
- Add transporter to inquiry detail ROW_OPTIONS and Services interface
- Archive resolved bug reports to bug_reports/resolved/
</commit_message>
<xml_diff>
--- a/templates/offer_template.xlsx
+++ b/templates/offer_template.xlsx
@@ -1294,29 +1294,6 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>- Kartons werden Vorzeitig Geliefert und Werden nach dem Umzug mit 2€ Je Woche berechnet</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
-            <a:effectLst/>
-            <a:uFillTx/>
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="de-DE" sz="1100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:uFillTx/>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
             <a:t>- Massive Holzmöbel / Designermöbel müssen gesondert benannt werden </a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">

</xml_diff>

<commit_message>
fix: auto-save multi-day employee time fields on blur, remove deprecated Planned fields
- Add normalizeTimeInput() to format.ts
- Remove deprecated 'Pl.' fields from multi-day views
- Auto-save clock_in/clock_out/break_minutes on blur via PATCH
- Clean up PUT bodies in save functions
</commit_message>
<xml_diff>
--- a/templates/offer_template.xlsx
+++ b/templates/offer_template.xlsx
@@ -3093,7 +3093,7 @@
         <v>28</v>
       </c>
       <c r="G38" s="62" t="n">
-        <f aca="false">IF(E38="", 0, F38*E38*J50)</f>
+        <f aca="false">IF(E38="", 0, F38*E38*J58)</f>
         <v>0</v>
       </c>
       <c r="I38" s="63"/>
@@ -3196,143 +3196,190 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="8"/>
-      <c r="B43" s="8"/>
-      <c r="C43" s="68"/>
-      <c r="D43" s="69"/>
-      <c r="E43" s="69"/>
-      <c r="F43" s="69"/>
-      <c r="G43" s="69"/>
-    </row>
-    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="8"/>
-      <c r="C44" s="70" t="s">
+    <row r="43" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="54"/>
+      <c r="B43" s="54"/>
+      <c r="C43" s="55"/>
+      <c r="D43" s="56"/>
+      <c r="E43" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="57" t="n">
+        <f aca="false">IF(E43="", 0, F43*E43)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="59"/>
+      <c r="B44" s="59"/>
+      <c r="C44" s="60"/>
+      <c r="D44" s="61"/>
+      <c r="E44" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="62" t="n">
+        <f aca="false">IF(E44="", 0, F44*E44)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="54"/>
+      <c r="B45" s="54"/>
+      <c r="C45" s="55"/>
+      <c r="D45" s="56"/>
+      <c r="E45" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="57" t="n">
+        <f aca="false">IF(E45="", 0, F45*E45)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="59"/>
+      <c r="B46" s="59"/>
+      <c r="C46" s="60"/>
+      <c r="D46" s="61"/>
+      <c r="E46" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="62" t="n">
+        <f aca="false">IF(E46="", 0, F46*E46)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="54"/>
+      <c r="B47" s="54"/>
+      <c r="C47" s="55"/>
+      <c r="D47" s="56"/>
+      <c r="E47" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="57" t="n">
+        <f aca="false">IF(E47="", 0, F47*E47)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="59"/>
+      <c r="B48" s="59"/>
+      <c r="C48" s="60"/>
+      <c r="D48" s="61"/>
+      <c r="E48" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="62" t="n">
+        <f aca="false">IF(E48="", 0, F48*E48)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="54"/>
+      <c r="B49" s="54"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="56"/>
+      <c r="E49" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="57" t="n">
+        <f aca="false">IF(E49="", 0, F49*E49)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="59"/>
+      <c r="B50" s="59"/>
+      <c r="C50" s="60"/>
+      <c r="D50" s="61"/>
+      <c r="E50" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="62" t="n">
+        <f aca="false">IF(E50="", 0, F50*E50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="8"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="68"/>
+      <c r="D51" s="69"/>
+      <c r="E51" s="69"/>
+      <c r="F51" s="69"/>
+      <c r="G51" s="69"/>
+    </row>
+    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="8"/>
+      <c r="C52" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="D44" s="69"/>
-      <c r="E44" s="71"/>
-      <c r="F44" s="71"/>
-      <c r="G44" s="72" t="n">
+      <c r="D52" s="69"/>
+      <c r="E52" s="71"/>
+      <c r="F52" s="71"/>
+      <c r="G52" s="72" t="n">
         <f aca="false">G31+G32+G33+G34+G35+G37+G38+G39+G41+G42+G40</f>
         <v>120</v>
       </c>
-      <c r="J44" s="53"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="8"/>
-      <c r="C45" s="70" t="s">
+      <c r="J52" s="53"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="8"/>
+      <c r="C53" s="70" t="s">
         <v>50</v>
       </c>
-      <c r="D45" s="69"/>
-      <c r="E45" s="71"/>
-      <c r="F45" s="71"/>
-      <c r="G45" s="72" t="n">
-        <f aca="false">G44*19%</f>
+      <c r="D53" s="69"/>
+      <c r="E53" s="71"/>
+      <c r="F53" s="71"/>
+      <c r="G53" s="72" t="n">
+        <f aca="false">G52*19%</f>
         <v>22.8</v>
       </c>
-      <c r="J45" s="53"/>
-      <c r="M45" s="73"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C46" s="1" t="s">
+      <c r="J53" s="53"/>
+      <c r="M53" s="73"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C54" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E46" s="74"/>
-      <c r="F46" s="74"/>
-      <c r="G46" s="75" t="n">
-        <f aca="false">G44+G45</f>
+      <c r="E54" s="74"/>
+      <c r="F54" s="74"/>
+      <c r="G54" s="75" t="n">
+        <f aca="false">G52+G53</f>
         <v>142.8</v>
       </c>
-      <c r="J46" s="53"/>
-      <c r="M46" s="73"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J47" s="53"/>
-      <c r="M47" s="73"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="47"/>
-      <c r="B48" s="47"/>
-      <c r="C48" s="47"/>
-      <c r="D48" s="47"/>
-      <c r="E48" s="47"/>
-      <c r="F48" s="47"/>
-      <c r="G48" s="47"/>
-      <c r="J48" s="53"/>
-      <c r="M48" s="73"/>
-    </row>
-    <row r="49" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="47"/>
-      <c r="B49" s="47"/>
-      <c r="C49" s="47"/>
-      <c r="D49" s="47"/>
-      <c r="E49" s="47"/>
-      <c r="F49" s="47"/>
-      <c r="G49" s="47"/>
-      <c r="J49" s="53"/>
-      <c r="M49" s="73"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="47"/>
-      <c r="B50" s="47"/>
-      <c r="C50" s="47"/>
-      <c r="D50" s="47"/>
-      <c r="E50" s="47"/>
-      <c r="F50" s="47"/>
-      <c r="G50" s="47"/>
-      <c r="J50" s="76"/>
-      <c r="M50" s="77"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="47"/>
-      <c r="B51" s="47"/>
-      <c r="C51" s="47"/>
-      <c r="D51" s="47"/>
-      <c r="E51" s="47"/>
-      <c r="F51" s="47"/>
-      <c r="G51" s="47"/>
-      <c r="J51" s="53"/>
-      <c r="M51" s="77"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47"/>
-      <c r="B52" s="47"/>
-      <c r="C52" s="47"/>
-      <c r="D52" s="47"/>
-      <c r="E52" s="47"/>
-      <c r="F52" s="47"/>
-      <c r="G52" s="47"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="47"/>
-      <c r="B53" s="47"/>
-      <c r="C53" s="47"/>
-      <c r="D53" s="47"/>
-      <c r="E53" s="47"/>
-      <c r="F53" s="47"/>
-      <c r="G53" s="47"/>
-    </row>
-    <row r="54" customFormat="false" ht="2.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="47"/>
-      <c r="B54" s="47"/>
-      <c r="C54" s="47"/>
-      <c r="D54" s="47"/>
-      <c r="E54" s="47"/>
-      <c r="F54" s="47"/>
-      <c r="G54" s="47"/>
+      <c r="J54" s="53"/>
+      <c r="M54" s="73"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="47"/>
-      <c r="B55" s="47"/>
-      <c r="C55" s="47"/>
-      <c r="D55" s="47"/>
-      <c r="E55" s="47"/>
-      <c r="F55" s="47"/>
-      <c r="G55" s="47"/>
-      <c r="J55" s="78"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J55" s="53"/>
+      <c r="M55" s="73"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="47"/>
       <c r="B56" s="47"/>
       <c r="C56" s="47"/>
@@ -3340,9 +3387,90 @@
       <c r="E56" s="47"/>
       <c r="F56" s="47"/>
       <c r="G56" s="47"/>
+      <c r="J56" s="53"/>
+      <c r="M56" s="73"/>
+    </row>
+    <row r="57" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="47"/>
+      <c r="B57" s="47"/>
+      <c r="C57" s="47"/>
+      <c r="D57" s="47"/>
+      <c r="E57" s="47"/>
+      <c r="F57" s="47"/>
+      <c r="G57" s="47"/>
+      <c r="J57" s="53"/>
+      <c r="M57" s="73"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="47"/>
+      <c r="B58" s="47"/>
+      <c r="C58" s="47"/>
+      <c r="D58" s="47"/>
+      <c r="E58" s="47"/>
+      <c r="F58" s="47"/>
+      <c r="G58" s="47"/>
+      <c r="J58" s="76"/>
+      <c r="M58" s="77"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="47"/>
+      <c r="B59" s="47"/>
+      <c r="C59" s="47"/>
+      <c r="D59" s="47"/>
+      <c r="E59" s="47"/>
+      <c r="F59" s="47"/>
+      <c r="G59" s="47"/>
+      <c r="J59" s="53"/>
+      <c r="M59" s="77"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="47"/>
+      <c r="B60" s="47"/>
+      <c r="C60" s="47"/>
+      <c r="D60" s="47"/>
+      <c r="E60" s="47"/>
+      <c r="F60" s="47"/>
+      <c r="G60" s="47"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="47"/>
+      <c r="B61" s="47"/>
+      <c r="C61" s="47"/>
+      <c r="D61" s="47"/>
+      <c r="E61" s="47"/>
+      <c r="F61" s="47"/>
+      <c r="G61" s="47"/>
+    </row>
+    <row r="62" customFormat="false" ht="2.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="47"/>
+      <c r="B62" s="47"/>
+      <c r="C62" s="47"/>
+      <c r="D62" s="47"/>
+      <c r="E62" s="47"/>
+      <c r="F62" s="47"/>
+      <c r="G62" s="47"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="47"/>
+      <c r="B63" s="47"/>
+      <c r="C63" s="47"/>
+      <c r="D63" s="47"/>
+      <c r="E63" s="47"/>
+      <c r="F63" s="47"/>
+      <c r="G63" s="47"/>
+      <c r="J63" s="78"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="47"/>
+      <c r="B64" s="47"/>
+      <c r="C64" s="47"/>
+      <c r="D64" s="47"/>
+      <c r="E64" s="47"/>
+      <c r="F64" s="47"/>
+      <c r="G64" s="47"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="46">
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
@@ -3368,7 +3496,7 @@
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A32:B32"/>
-    <mergeCell ref="I32:M41"/>
+    <mergeCell ref="I32:M49"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="A37:B37"/>
@@ -3376,11 +3504,19 @@
     <mergeCell ref="A39:B39"/>
     <mergeCell ref="A41:B41"/>
     <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A48:G49"/>
-    <mergeCell ref="A50:G56"/>
+    <mergeCell ref="A56:G57"/>
+    <mergeCell ref="A58:G64"/>
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E18" r:id="rId1" display="E-Mail: "/>

</xml_diff>

<commit_message>
chore: snapshot in-progress backend work
Working-tree state committed as-is: DB-backed Stundensatz in offer line
items, Schlussrechnung rounding adjustment
(adjust_final_deduction_for_rounding), calendar/employee repo and
assistant tool updates, sqlx::test DB tests for flash-contact reminders,
backfill_end_date migration re-dated to 20260611 (was back-dated and
broke fresh DBs), offer template tweak, frontend submodule bump
(review fixes, version-skew fix, unit + integration test suites).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/offer_template.xlsx
+++ b/templates/offer_template.xlsx
@@ -542,7 +542,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="88">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -882,6 +882,10 @@
     </xf>
     <xf numFmtId="172" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
@@ -966,13 +970,13 @@
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>797040</xdr:colOff>
+      <xdr:colOff>925056</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>79560</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>704160</xdr:colOff>
+      <xdr:colOff>832176</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>185040</xdr:rowOff>
     </xdr:to>
@@ -2239,19 +2243,14 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>434880</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>95400</xdr:rowOff>
+      <xdr:colOff>638266</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>169284</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>545400</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>38520</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="2500000" cy="1653578"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Grafik 2"/>
@@ -2264,7 +2263,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5200560" y="371520"/>
-          <a:ext cx="2419200" cy="1574640"/>
+          <a:ext cx="2500000" cy="1653578"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2276,7 +2275,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2473,7 +2472,11 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Aust Umzüge und Haushaltsauflösungen</t>
+        </is>
+      </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2481,7 +2484,11 @@
       <c r="F2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Ihr Umzug in besten Händen bei Aust!</t>
+        </is>
+      </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>

</xml_diff>

<commit_message>
fix(offers): wrap long KVA Bemerkung text and grow row height
Long remark text in column C of the offer XLSX overflowed instead of
wrapping, since only the short-remark cell style existed. Adds a
wrap-enabled style pair and estimates the wrapped line count to grow
the row height accordingly, so multi-line remarks (e.g. insurance
coverage notes) render fully.
</commit_message>
<xml_diff>
--- a/templates/offer_template.xlsx
+++ b/templates/offer_template.xlsx
@@ -542,7 +542,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="90">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -885,6 +885,14 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
fix(kva): size the terms-page signature lines to the box that holds them
The signature line still wrapped into two stacked rules on the Umzug terms page.
Installing Carlito was necessary but not sufficient: the drawing's text box
renders ~376-386pt wide, not the ~436pt its <a:ext cx> implies, and the
96-character line measures 415.7pt in Carlito at 11pt.

Sized both blocks against the real box width using Carlito metrics: 23
underscores + 23 spaces + 28 underscores (336.6pt), with the second group
starting under "Datum, Unterschrift Umzugsunternehmen". Verified by converting
the template with LibreOffice inside the deployed backend image.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ug2cocAJTqVwGFvZz8qrND
</commit_message>
<xml_diff>
--- a/templates/offer_template.xlsx
+++ b/templates/offer_template.xlsx
@@ -1812,7 +1812,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>_______________________                                   _____________________________________</a:t>
+            <a:t>_______________________                       ____________________________</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="de-DE" sz="1100" b="0" u="none" strike="noStrike">
@@ -2161,7 +2161,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>_______________________                                   _____________________________________ </a:t>
+            <a:t>_______________________                       ____________________________ </a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>

</xml_diff>

<commit_message>
fix(kva): shrink the letterhead logo so it stops being clipped
The logo is anchored to a spreadsheet column plus an offset, so where it
lands depends on the renderer's column widths. In the production image
Calibri falls back to Carlito, the columns come out wider, and the picture
was pushed past the right print margin — customers received KVAs reading
"Aust Umzüg". The host's LibreOffice never showed it.

Keep the anchor exactly where it was and only reduce the picture, 2.5M to
2.0M EMU wide at the same aspect ratio. The rendered logo now keeps ~8mm
of clearance to the print margin.

check-templates.py grows a check for this: it rasterises page 1, finds the
logo as the only coloured element in the top quarter, and fails unless its
right edge stays 8pt clear of the margin. Verified to fail on the old size.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016GeSo2pPmBp5EyZdEGXPMS
</commit_message>
<xml_diff>
--- a/templates/offer_template.xlsx
+++ b/templates/offer_template.xlsx
@@ -2221,7 +2221,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>169284</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2500000" cy="1653578"/>
+    <xdr:ext cx="2000000" cy="1322862"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Grafik 2"/>
@@ -2234,7 +2234,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5200560" y="371520"/>
-          <a:ext cx="2500000" cy="1653578"/>
+          <a:ext cx="2000000" cy="1322862"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>